<commit_message>
F9, F14a, N62, N27
</commit_message>
<xml_diff>
--- a/Docs/AI/Polls/2026-10-24_Poll-Report15.xlsx
+++ b/Docs/AI/Polls/2026-10-24_Poll-Report15.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Lesson\FallenStar-Spellcasters\Docs\AI\Polls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6BA8D42-FF28-4ED8-B5BB-D2BA7C798765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1B56CBE-9057-4AC1-AF17-8FB177989FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="6135" windowWidth="38400" windowHeight="17145" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read me" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="156">
   <si>
     <t>Priorities: feature gaps (not defects). Pre-filled with your 2026-10-24 ranking; change any of them.</t>
   </si>
@@ -482,6 +482,46 @@
   </si>
   <si>
     <t>Can you please sort futures by priority in this poll next time? It's kinda hard to navigate, so</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Moving animation + rotation</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Delegate to other claude agent to create animation for current character model</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Later</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Reposition of game scene</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Reposition of whole game scene to improve visuability. For example, focus camera only on player side of desc, only on enemy side, general plan</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Add some animation to card</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Add animation on card click/selection on local machine and general animation for each player (explosions/magic/etc). Need some research, I'll give you some assets for research.</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Animation setting</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>2 setting for focus camera on current player movement or card target or leave it free(to change between free camera, enemy zoom, self zoom), separate 2 setting - showing hint about what how to play current selected card and auto select zoom on possible target(additional switch for cases - do ... to ANY player character/Block/Random for both team)</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>Later, when general animation system will be done for tests</t>
     <phoneticPr fontId="9"/>
   </si>
 </sst>
@@ -1464,7 +1504,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1804,8 +1844,52 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="38.25" x14ac:dyDescent="0.15">
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="2" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B24" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="C24" t="s">
+        <v>147</v>
+      </c>
+      <c r="E24" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B25" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="C25" t="s">
+        <v>150</v>
+      </c>
+      <c r="E25" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B26" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="C26" t="s">
+        <v>152</v>
+      </c>
+      <c r="E26" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B27" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="C27" t="s">
+        <v>154</v>
+      </c>
+      <c r="E27" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>